<commit_message>
Implement requested PMS updates across modules.
Apply customer, transfer, property, project, payment plan, migration, and SQL dump workflow changes requested for deployment readiness.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PMS/wwwroot/samples/property.xlsx
+++ b/PMS/wwwroot/samples/property.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -16,20 +16,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="31">
-  <si>
-    <t>Apartment</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="27">
   <si>
     <t>Street</t>
   </si>
   <si>
-    <t>Block</t>
-  </si>
-  <si>
-    <t>PropertyType</t>
-  </si>
-  <si>
     <t>Size</t>
   </si>
   <si>
@@ -81,12 +72,6 @@
     <t>2476.03 Sq Ft</t>
   </si>
   <si>
-    <t>SubProject</t>
-  </si>
-  <si>
-    <t>ZKB Eclipse</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -109,12 +94,15 @@
   </si>
   <si>
     <t>Unit No</t>
+  </si>
+  <si>
+    <t>Tower or Block</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -172,6 +160,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
@@ -219,7 +210,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -254,7 +245,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -463,302 +454,236 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.140625" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.28515625" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.28515625" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="D4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="B6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="B7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="C9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="C11" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+        <v>14</v>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>